<commit_message>
final code with images and excel automattion
</commit_message>
<xml_diff>
--- a/models_master.xlsx
+++ b/models_master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yuckq\Desktop\amazon screipts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B257E3CD-0AB2-48AB-A002-F43B7EC5EB0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C8A20F6-F087-479D-AD48-530B3B629045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2295" yWindow="2295" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="44">
   <si>
     <t>model_key</t>
   </si>
@@ -148,25 +148,7 @@
     <t>iPhone_17</t>
   </si>
   <si>
-    <t>iPhone_18</t>
-  </si>
-  <si>
-    <t>iPhone_19</t>
-  </si>
-  <si>
-    <t>iPhone_20</t>
-  </si>
-  <si>
     <t>Yuckquee Compatible with iPhone 17 Mobile Skin /Wrap/Sticker for Back &amp; Camera Protective, Stratchless, Matte.</t>
-  </si>
-  <si>
-    <t>Yuckquee Compatible with iPhone 18 Mobile Skin /Wrap/Sticker for Back &amp; Camera Protective, Stratchless, Matte.</t>
-  </si>
-  <si>
-    <t>Yuckquee Compatible with iPhone 19 Mobile Skin /Wrap/Sticker for Back &amp; Camera Protective, Stratchless, Matte.</t>
-  </si>
-  <si>
-    <t>Yuckquee Compatible with iPhone 20 Mobile Skin /Wrap/Sticker for Back &amp; Camera Protective, Stratchless, Matte.</t>
   </si>
   <si>
     <t>num_designs</t>
@@ -517,7 +499,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AN5"/>
+  <dimension ref="A1:AN2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:40" x14ac:dyDescent="0.25">
@@ -537,7 +519,7 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="G1" t="s">
         <v>0</v>
@@ -650,7 +632,7 @@
         <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D2">
         <v>24</v>
@@ -668,93 +650,6 @@
         <v>39</v>
       </c>
       <c r="U2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3">
-        <v>24</v>
-      </c>
-      <c r="F3">
-        <v>123</v>
-      </c>
-      <c r="G3" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>38</v>
-      </c>
-      <c r="R3" t="s">
-        <v>39</v>
-      </c>
-      <c r="U3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="4" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D4">
-        <v>24</v>
-      </c>
-      <c r="F4">
-        <v>123</v>
-      </c>
-      <c r="G4" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>38</v>
-      </c>
-      <c r="R4" t="s">
-        <v>39</v>
-      </c>
-      <c r="U4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D5">
-        <v>24</v>
-      </c>
-      <c r="F5">
-        <v>123</v>
-      </c>
-      <c r="G5" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>38</v>
-      </c>
-      <c r="R5" t="s">
-        <v>39</v>
-      </c>
-      <c r="U5" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>